<commit_message>
anpassungen sim an den metadaten zu den brunnenfotos
</commit_message>
<xml_diff>
--- a/automation/wvz_brunnenbilder/meta_wvz_brunnenbilder.xlsx
+++ b/automation/wvz_brunnenbilder/meta_wvz_brunnenbilder.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sszgua\Python\jupyter\ogd\brunnen\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\sszsim\1_github_odz\opendatazurich.github.io\automation\wvz_brunnenbilder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11D08E43-108D-4C8D-9C96-7C167EA6E5A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{094A7B1E-8E0C-4844-86C5-2888E8D99944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="21860" yWindow="2660" windowWidth="30330" windowHeight="10780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="metadata" sheetId="14" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="180">
   <si>
     <t>Tagname</t>
   </si>
@@ -942,21 +942,9 @@
     <t>Datenerhebung:</t>
   </si>
   <si>
-    <t>01.06.2026</t>
-  </si>
-  <si>
     <t>Datenquelle:</t>
   </si>
   <si>
-    <t>Brunnenbilder</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Bauen und Wohnen,  Verwaltung</t>
-  </si>
-  <si>
-    <t>brunnen, wasserversorgung, bilder</t>
-  </si>
-  <si>
     <t>Statistik Stadt Zürich, Präsidialdepartement</t>
   </si>
   <si>
@@ -984,19 +972,34 @@
     <t>Direktlink zum Bild des Brunnens</t>
   </si>
   <si>
-    <t>Die Bild-URLs werden von den Unterseiten der [Brunnen Webseite](https://www.stadt-zuerich.ch/de/umwelt-und-energie/wasser/trinkwasser/brunnen.html) übernommen.</t>
-  </si>
-  <si>
     <t>bild_url</t>
   </si>
   <si>
     <t>brunnennummer</t>
   </si>
   <si>
-    <t>Dieser Datensatz ist eine Ergänzung zum [Geodatensatz mit den Brunnen der Stadt Zürich](https://data.stadt-zuerich.ch/dataset/geo_brunnen). Er sammelt die URLs der [Brunnenwebseite](https://www.stadt-zuerich.ch/de/umwelt-und-energie/wasser/trinkwasser/brunnen.html) und der zugehörigen Bilder. Über die Brunnennummer können diese Informationen mit dem Geodatensatz verknüpft werden.</t>
-  </si>
-  <si>
-    <t>Im [Geodatensatz mit den Brunnen](https://data.stadt-zuerich.ch/dataset/geo_brunnen) sind URLs zu Bildern der einzelnen Brunnen enthalten. Diese URLs sind aus Urheberrechtsgründen nicht frei zugänglich. Die Stadt Zürich publiziert aber auf dieser [Webseite](https://www.stadt-zuerich.ch/de/umwelt-und-energie/wasser/trinkwasser/brunnen.html) Informationen zu den einzelnen Brunnen. In vielen Fällen ist auch ein Bild davon verfügbar. Dieser Datensatz sammelt die URLs der Brunnenwebseite und der zugehörigen Bilder per Webscraping.</t>
+    <t>Brunnenfotos der Stadt Zürich</t>
+  </si>
+  <si>
+    <t>Dieser Datensatz ergänzt den [Geodatensatz mit den Brunnen der Stadt Zürich](https://data.stadt-zuerich.ch/dataset/geo_brunnen). Er enthält die URLs der öffentlich zugänglichen [Brunnenwebseiten](https://www.stadt-zuerich.ch/de/umwelt-und-energie/wasser/trinkwasser/brunnen.html) sowie der zugehörigen Fotos. Über die Brunnennummer lassen sich diese Informationen mit dem Geodatensatz verknüpfen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Bauen und Wohnen,  Verwaltung, Gesundheit</t>
+  </si>
+  <si>
+    <t>Aktuelles Datum</t>
+  </si>
+  <si>
+    <t>13.05.2026</t>
+  </si>
+  <si>
+    <t>brunnen, wasserversorgung, bilder, fotos, trinkwasser</t>
+  </si>
+  <si>
+    <t>Die Bild-URLs werden von den Unterseiten der [Brunnen-Webseite](https://www.stadt-zuerich.ch/de/umwelt-und-energie/wasser/trinkwasser/brunnen.html) übernommen.</t>
+  </si>
+  <si>
+    <t>Der [Geodatensatz mit den Brunnen] (https://data.stadt-zuerich.ch/dataset/geo_brunnen) enthält zwar URLs zu Fotos der einzelnen Brunnen, diese sind jedoch nicht öffentlich zugänglich. Auf der [Brunnen-Webseite] (https://www.stadt-zuerich.ch/de/umwelt-und-energie/wasser/trinkwasser/brunnen.html) publiziert die Stadt Zürich hingegen frei zugängliche Informationen und vielfach auch Fotos zu den einzelnen Brunnen. Der vorliegende Datensatz bezieht die URLs dieser Webseiten und der zugehörigen Fotos per Webscraping.</t>
   </si>
 </sst>
 </file>
@@ -1720,20 +1723,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="255.5" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:G33"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="255.5" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.125" style="11" customWidth="1"/>
+    <col min="1" max="1" width="14.08203125" style="11" customWidth="1"/>
     <col min="2" max="2" width="24.5" style="4" customWidth="1"/>
-    <col min="3" max="3" width="66.875" style="4" customWidth="1"/>
-    <col min="4" max="4" width="53.625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="66.83203125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="53.58203125" style="5" customWidth="1"/>
     <col min="5" max="5" width="8.75" style="5" customWidth="1"/>
-    <col min="6" max="6" width="88.875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="50.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="88.83203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="50.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="255.5" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -1756,7 +1759,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="4" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" s="4" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
         <v>7</v>
       </c>
@@ -1767,14 +1770,14 @@
         <v>9</v>
       </c>
       <c r="D2" s="22" t="s">
-        <v>162</v>
+        <v>172</v>
       </c>
       <c r="E2" s="7"/>
       <c r="F2" s="7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:7" s="4" customFormat="1" ht="89.25" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" s="4" customFormat="1" ht="91" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
         <v>11</v>
       </c>
@@ -1785,14 +1788,14 @@
         <v>9</v>
       </c>
       <c r="D3" s="34" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="E3" s="7"/>
       <c r="F3" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:7" s="4" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" s="4" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
         <v>14</v>
       </c>
@@ -1803,14 +1806,14 @@
         <v>9</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:7" s="4" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" s="4" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
         <v>17</v>
       </c>
@@ -1826,7 +1829,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:7" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
         <v>21</v>
       </c>
@@ -1844,7 +1847,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:7" s="4" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" s="4" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
         <v>24</v>
       </c>
@@ -1855,14 +1858,14 @@
         <v>9</v>
       </c>
       <c r="D7" s="34" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="E7" s="7"/>
       <c r="F7" s="8" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:7" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>27</v>
       </c>
@@ -1873,14 +1876,14 @@
         <v>9</v>
       </c>
       <c r="D8" s="34" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E8" s="7"/>
       <c r="F8" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:7" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>30</v>
       </c>
@@ -1891,14 +1894,14 @@
         <v>9</v>
       </c>
       <c r="D9" s="34" t="s">
-        <v>115</v>
+        <v>175</v>
       </c>
       <c r="E9" s="7"/>
       <c r="F9" s="7" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:7" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
         <v>33</v>
       </c>
@@ -1914,7 +1917,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:7" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>36</v>
       </c>
@@ -1925,14 +1928,14 @@
         <v>19</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
       <c r="E11" s="9"/>
       <c r="F11" s="7" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:7" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
         <v>39</v>
       </c>
@@ -1942,13 +1945,15 @@
       <c r="C12" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="19"/>
+      <c r="D12" s="19" t="s">
+        <v>48</v>
+      </c>
       <c r="E12" s="9"/>
       <c r="F12" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:7" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
         <v>42</v>
       </c>
@@ -1966,7 +1971,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:7" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
         <v>46</v>
       </c>
@@ -1984,7 +1989,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="15" spans="1:7" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
         <v>50</v>
       </c>
@@ -1995,14 +2000,14 @@
         <v>9</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
       <c r="E15" s="7"/>
       <c r="F15" s="7" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="16" spans="1:7" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
         <v>53</v>
       </c>
@@ -2020,7 +2025,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="17" spans="1:6" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A17" s="33" t="s">
         <v>56</v>
       </c>
@@ -2038,14 +2043,14 @@
         <v>59</v>
       </c>
     </row>
-    <row r="18" spans="1:6" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A18" s="11"/>
       <c r="B18" s="3"/>
       <c r="C18" s="7"/>
       <c r="E18" s="7"/>
       <c r="F18" s="7"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
         <v>60</v>
       </c>
@@ -2058,7 +2063,7 @@
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B20" s="13" t="s">
         <v>8</v>
       </c>
@@ -2068,169 +2073,163 @@
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
     </row>
-    <row r="21" spans="1:6" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" ht="37.5" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
         <v>62</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C21" s="35" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
-    </row>
-    <row r="22" spans="1:6" ht="89.25" x14ac:dyDescent="0.2">
+      <c r="F21" s="8" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="87.5" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
         <v>62</v>
       </c>
       <c r="B22" s="21" t="s">
         <v>159</v>
       </c>
-      <c r="C22" s="35" t="s">
-        <v>178</v>
+      <c r="C22" s="21" t="s">
+        <v>179</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="7"/>
-      <c r="F22" s="8" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="43.5" x14ac:dyDescent="0.2">
+      <c r="F22" s="23" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B23" s="21"/>
       <c r="C23" s="21"/>
       <c r="D23" s="1"/>
       <c r="E23" s="7"/>
-      <c r="F23" s="23" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B24" s="21"/>
-      <c r="C24" s="21"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B24" s="12"/>
+      <c r="C24" s="12"/>
       <c r="D24" s="1"/>
       <c r="E24" s="7"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B25" s="12"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="7"/>
-    </row>
-    <row r="26" spans="1:6" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A26" s="11"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="7"/>
-    </row>
-    <row r="27" spans="1:6" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A27" s="11" t="s">
+    <row r="25" spans="1:6" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A25" s="11"/>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="7"/>
+    </row>
+    <row r="26" spans="1:6" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A26" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B26" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C26" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="D26" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9" t="s">
+      <c r="E26" s="9"/>
+      <c r="F26" s="9" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="28" spans="1:6" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A28" s="11"/>
-      <c r="B28" s="13" t="s">
+    <row r="27" spans="1:6" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A27" s="11"/>
+      <c r="B27" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="C28" s="13" t="s">
+      <c r="C27" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="D28" s="13" t="s">
+      <c r="D27" s="13" t="s">
         <v>70</v>
+      </c>
+      <c r="E27" s="7"/>
+      <c r="F27" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A28" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="B28" s="21" t="s">
+        <v>171</v>
+      </c>
+      <c r="C28" s="21" t="s">
+        <v>164</v>
+      </c>
+      <c r="D28" s="21" t="s">
+        <v>163</v>
       </c>
       <c r="E28" s="7"/>
       <c r="F28" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" s="4" customFormat="1" ht="25" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
         <v>72</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="C29" s="21" t="s">
+        <v>166</v>
+      </c>
+      <c r="D29" s="21" t="s">
         <v>168</v>
-      </c>
-      <c r="D29" s="21" t="s">
-        <v>167</v>
       </c>
       <c r="E29" s="7"/>
       <c r="F29" s="4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" s="4" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" s="4" customFormat="1" ht="12.5" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
         <v>72</v>
       </c>
       <c r="B30" s="21" t="s">
+        <v>170</v>
+      </c>
+      <c r="C30" s="21" t="s">
+        <v>167</v>
+      </c>
+      <c r="D30" s="21" t="s">
         <v>169</v>
       </c>
-      <c r="C30" s="21" t="s">
-        <v>170</v>
-      </c>
-      <c r="D30" s="21" t="s">
-        <v>172</v>
-      </c>
       <c r="E30" s="7"/>
-      <c r="F30" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A31" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="B31" s="21" t="s">
-        <v>175</v>
-      </c>
-      <c r="C31" s="21" t="s">
-        <v>171</v>
-      </c>
-      <c r="D31" s="21" t="s">
-        <v>173</v>
-      </c>
+    </row>
+    <row r="31" spans="1:6" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A31" s="11"/>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="7"/>
       <c r="E31" s="7"/>
     </row>
-    <row r="32" spans="1:6" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A32" s="11"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
       <c r="D32" s="7"/>
       <c r="E32" s="7"/>
     </row>
-    <row r="33" spans="1:5" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A33" s="11"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
       <c r="D33" s="7"/>
       <c r="E33" s="7"/>
-    </row>
-    <row r="34" spans="1:5" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A34" s="11"/>
-      <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="7"/>
-      <c r="E34" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.98425196850393704" bottom="0.59055118110236227" header="0.39370078740157483" footer="0.27559055118110237"/>
@@ -2241,131 +2240,131 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.375" style="24" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.33203125" style="24" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.25" style="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.625" style="24" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.875" style="24" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.625" style="24" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.375" style="24" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.125" style="24" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.375" style="24" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.875" style="24" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.625" style="24" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.375" style="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.58203125" style="24" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.83203125" style="24" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.58203125" style="24" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.33203125" style="24" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.08203125" style="24" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.33203125" style="24" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.83203125" style="24" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.58203125" style="24" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.33203125" style="24" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8.75" style="24" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.625" style="24" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.875" style="24" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.58203125" style="24" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.83203125" style="24" bestFit="1" customWidth="1"/>
     <col min="15" max="16384" width="11" style="24"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="25" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A2" s="29" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A3" s="29" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A4" s="29" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A5" s="29" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A6" s="29" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A7" s="29" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A8" s="29" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A9" s="29" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A10" s="29" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A11" s="29" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A12" s="29" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A13" s="29" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A14" s="29" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A15" s="29" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="16" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A16" s="29" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A17" s="29" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A18" s="29" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A19" s="29" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="20" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A20" s="29" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" s="31" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" s="32" t="s">
         <v>96</v>
       </c>
@@ -2382,14 +2381,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.5" style="24" customWidth="1"/>
-    <col min="2" max="2" width="5.625" style="24" customWidth="1"/>
+    <col min="2" max="2" width="5.58203125" style="24" customWidth="1"/>
     <col min="3" max="16384" width="11" style="24"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="25" t="s">
         <v>75</v>
       </c>
@@ -2397,27 +2396,27 @@
         <v>97</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A2" s="29" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A3" s="29" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A4" s="29" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A5" s="29" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A6" s="30" t="s">
         <v>101</v>
       </c>
@@ -2425,12 +2424,12 @@
         <v>102</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="31" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="32" t="s">
         <v>96</v>
       </c>
@@ -2447,14 +2446,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="35.375" style="24" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.33203125" style="24" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.25" style="24" customWidth="1"/>
     <col min="3" max="16384" width="11" style="24"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="25" t="s">
         <v>75</v>
       </c>
@@ -2462,118 +2461,118 @@
         <v>97</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A2" s="29" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A3" s="29" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A4" s="29" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A5" s="29" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A6" s="29" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A7" s="29" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A8" s="29" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A9" s="29" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A10" s="29" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A11" s="29" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A12" s="29" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A13" s="29" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A14" s="29" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A15" s="29" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A16" s="29" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A17" s="30" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A18" s="26"/>
     </row>
-    <row r="19" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A19" s="26"/>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="31" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" s="32" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="22" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A22" s="26"/>
     </row>
-    <row r="23" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A23" s="26"/>
     </row>
-    <row r="24" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A24" s="26"/>
     </row>
-    <row r="25" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A25" s="26"/>
     </row>
-    <row r="26" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A26" s="26"/>
     </row>
-    <row r="27" spans="1:1" ht="15" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:1" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A27" s="26"/>
     </row>
   </sheetData>
@@ -2588,15 +2587,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.5" style="24" customWidth="1"/>
-    <col min="2" max="2" width="5.375" style="24" customWidth="1"/>
-    <col min="3" max="3" width="58.625" style="24" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.33203125" style="24" customWidth="1"/>
+    <col min="3" max="3" width="58.58203125" style="24" bestFit="1" customWidth="1"/>
     <col min="4" max="16384" width="11" style="24"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="25" t="s">
         <v>75</v>
       </c>
@@ -2607,7 +2606,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A2" s="29" t="s">
         <v>119</v>
       </c>
@@ -2619,7 +2618,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A3" s="29" t="s">
         <v>122</v>
       </c>
@@ -2631,7 +2630,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A4" s="29" t="s">
         <v>125</v>
       </c>
@@ -2643,7 +2642,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A5" s="29" t="s">
         <v>128</v>
       </c>
@@ -2655,7 +2654,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A6" s="27" t="s">
         <v>58</v>
       </c>
@@ -2667,7 +2666,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A7" s="27" t="s">
         <v>133</v>
       </c>
@@ -2679,7 +2678,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A8" s="27" t="s">
         <v>136</v>
       </c>
@@ -2691,7 +2690,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A9" s="29" t="s">
         <v>139</v>
       </c>
@@ -2703,7 +2702,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A10" s="29" t="s">
         <v>142</v>
       </c>
@@ -2715,7 +2714,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A11" s="29" t="s">
         <v>144</v>
       </c>
@@ -2727,7 +2726,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A12" s="29" t="s">
         <v>146</v>
       </c>
@@ -2739,7 +2738,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A13" s="29" t="s">
         <v>148</v>
       </c>
@@ -2751,7 +2750,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A14" s="29" t="s">
         <v>151</v>
       </c>
@@ -2763,7 +2762,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A15" s="29" t="s">
         <v>154</v>
       </c>
@@ -2775,7 +2774,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A16" s="29" t="s">
         <v>156</v>
       </c>
@@ -2787,12 +2786,12 @@
         <v>121</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="31" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" ht="14.5" x14ac:dyDescent="0.3">
       <c r="A22" s="32" t="s">
         <v>96</v>
       </c>
@@ -2808,26 +2807,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="637d3f4c-beee-42dd-a17b-93f7589025e5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="31d8624d-d3e1-4449-addd-518bfa42d279">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010036EB69643BC4D84A90CF31D6917ED8B0" ma:contentTypeVersion="17" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="e787fa9c9cb978e1d00e8cc5d4e605d2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="31d8624d-d3e1-4449-addd-518bfa42d279" xmlns:ns3="637d3f4c-beee-42dd-a17b-93f7589025e5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="369004915ca410f163a62304f925ff92" ns2:_="" ns3:_="">
     <xsd:import namespace="31d8624d-d3e1-4449-addd-518bfa42d279"/>
@@ -3076,10 +3055,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="637d3f4c-beee-42dd-a17b-93f7589025e5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="31d8624d-d3e1-4449-addd-518bfa42d279">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4B3AD83-9986-4E71-995F-A94C1CED6EB8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B249E2D-022F-440D-B037-6C32F5252DA3}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="31d8624d-d3e1-4449-addd-518bfa42d279"/>
+    <ds:schemaRef ds:uri="637d3f4c-beee-42dd-a17b-93f7589025e5"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3102,20 +3112,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B249E2D-022F-440D-B037-6C32F5252DA3}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4B3AD83-9986-4E71-995F-A94C1CED6EB8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="31d8624d-d3e1-4449-addd-518bfa42d279"/>
-    <ds:schemaRef ds:uri="637d3f4c-beee-42dd-a17b-93f7589025e5"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>